<commit_message>
Empaquetado en ejecutable con PyInstaller
</commit_message>
<xml_diff>
--- a/FormatoIngresoFactura.xlsx
+++ b/FormatoIngresoFactura.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanp\Documents\Codigo\Ingreso_automatico_facturas_compra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2F3D8A-9A35-4E70-9C7D-34DD08814CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{700515B9-1253-40F6-A54A-ECA844C8648E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{67A17E71-2B54-422E-9EB1-F47E5F398318}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="100">
   <si>
     <t>Fecha</t>
   </si>
@@ -59,39 +59,9 @@
     <t>3</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
-    <t>FC</t>
-  </si>
-  <si>
-    <t>04P023</t>
-  </si>
-  <si>
-    <t>01P925</t>
-  </si>
-  <si>
-    <t>FUS</t>
-  </si>
-  <si>
-    <t>8739</t>
-  </si>
-  <si>
-    <t>10588</t>
-  </si>
-  <si>
-    <t>10504</t>
-  </si>
-  <si>
-    <t>10420</t>
-  </si>
-  <si>
-    <t>115971</t>
-  </si>
-  <si>
     <t>DATOS FACTURA</t>
   </si>
   <si>
@@ -113,7 +83,262 @@
     <t>IVA</t>
   </si>
   <si>
-    <t>103250</t>
+    <t>BOG</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>29700</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>26000</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>FEV</t>
+  </si>
+  <si>
+    <t>62649</t>
+  </si>
+  <si>
+    <t>830021100</t>
+  </si>
+  <si>
+    <t>02R323</t>
+  </si>
+  <si>
+    <t>01R291</t>
+  </si>
+  <si>
+    <t>01R572</t>
+  </si>
+  <si>
+    <t>02R339</t>
+  </si>
+  <si>
+    <t>01R034</t>
+  </si>
+  <si>
+    <t>01R037</t>
+  </si>
+  <si>
+    <t>02T317</t>
+  </si>
+  <si>
+    <t>02T318</t>
+  </si>
+  <si>
+    <t>01T069</t>
+  </si>
+  <si>
+    <t>02T063</t>
+  </si>
+  <si>
+    <t>01T766</t>
+  </si>
+  <si>
+    <t>01T533</t>
+  </si>
+  <si>
+    <t>02T398</t>
+  </si>
+  <si>
+    <t>01B603</t>
+  </si>
+  <si>
+    <t>02T104</t>
+  </si>
+  <si>
+    <t>02T385</t>
+  </si>
+  <si>
+    <t>04B741</t>
+  </si>
+  <si>
+    <t>03T541</t>
+  </si>
+  <si>
+    <t>02T576</t>
+  </si>
+  <si>
+    <t>01T423</t>
+  </si>
+  <si>
+    <t>01T418</t>
+  </si>
+  <si>
+    <t>01T049</t>
+  </si>
+  <si>
+    <t>01T048</t>
+  </si>
+  <si>
+    <t>01T047</t>
+  </si>
+  <si>
+    <t>02T097</t>
+  </si>
+  <si>
+    <t>01T165</t>
+  </si>
+  <si>
+    <t>01R521</t>
+  </si>
+  <si>
+    <t>01R532</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>37900</t>
+  </si>
+  <si>
+    <t>30700</t>
+  </si>
+  <si>
+    <t>30900</t>
+  </si>
+  <si>
+    <t>26800</t>
+  </si>
+  <si>
+    <t>36270</t>
+  </si>
+  <si>
+    <t>40000</t>
+  </si>
+  <si>
+    <t>24300</t>
+  </si>
+  <si>
+    <t>27300</t>
+  </si>
+  <si>
+    <t>45000</t>
+  </si>
+  <si>
+    <t>32130</t>
+  </si>
+  <si>
+    <t>35900</t>
+  </si>
+  <si>
+    <t>34700</t>
+  </si>
+  <si>
+    <t>35000</t>
+  </si>
+  <si>
+    <t>37700</t>
+  </si>
+  <si>
+    <t>44300</t>
+  </si>
+  <si>
+    <t>29500</t>
+  </si>
+  <si>
+    <t>30400</t>
+  </si>
+  <si>
+    <t>33900</t>
+  </si>
+  <si>
+    <t>33000</t>
+  </si>
+  <si>
+    <t>35600</t>
+  </si>
+  <si>
+    <t>31300</t>
+  </si>
+  <si>
+    <t>29900</t>
+  </si>
+  <si>
+    <t>36000</t>
+  </si>
+  <si>
+    <t>34800</t>
+  </si>
+  <si>
+    <t>9.79</t>
+  </si>
+  <si>
+    <t>01R479</t>
+  </si>
+  <si>
+    <t>01T628</t>
+  </si>
+  <si>
+    <t>02T908</t>
+  </si>
+  <si>
+    <t>01T629</t>
+  </si>
+  <si>
+    <t>02R510</t>
+  </si>
+  <si>
+    <t>01B951</t>
+  </si>
+  <si>
+    <t>01A410</t>
+  </si>
+  <si>
+    <t>02B151</t>
+  </si>
+  <si>
+    <t>01V042</t>
+  </si>
+  <si>
+    <t>02T488</t>
+  </si>
+  <si>
+    <t>01T424</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>39900</t>
+  </si>
+  <si>
+    <t>35700</t>
+  </si>
+  <si>
+    <t>38900</t>
+  </si>
+  <si>
+    <t>30500</t>
+  </si>
+  <si>
+    <t>39000</t>
+  </si>
+  <si>
+    <t>21600</t>
+  </si>
+  <si>
+    <t>29771</t>
+  </si>
+  <si>
+    <t>42000</t>
   </si>
 </sst>
 </file>
@@ -208,10 +433,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -552,7 +777,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9761A0BD-3A6E-4B42-BA50-BD0DC4B983CA}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="2" customWidth="1"/>
@@ -562,65 +787,65 @@
     <col min="6" max="6" width="10.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" spans="1:6" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+    <row r="1" spans="1:10" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+    </row>
+    <row r="2" spans="1:10" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>46272</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>18</v>
-      </c>
       <c r="B4" s="5" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
@@ -628,103 +853,807 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J6">
+        <f>66423600/6784824</f>
+        <v>9.7900255039777004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="D23" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="D29" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="D30" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="D32" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="D36" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="D44" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F45" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualización de versión de software, por lo que se necesitó actualizar coordenadas
</commit_message>
<xml_diff>
--- a/FormatoIngresoFactura.xlsx
+++ b/FormatoIngresoFactura.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanp\Documents\Codigo\Ingreso_automatico_facturas_compra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDFFE09D-DBF3-4D8A-BD05-40FD63E25ADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78535879-FC9B-436D-91BA-64B0C257F502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{67A17E71-2B54-422E-9EB1-F47E5F398318}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{67A17E71-2B54-422E-9EB1-F47E5F398318}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="68">
   <si>
     <t>Fecha</t>
   </si>
@@ -95,79 +95,154 @@
     <t>1</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>02B466</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>32560</t>
-  </si>
-  <si>
-    <t>FEY</t>
-  </si>
-  <si>
-    <t>139092</t>
-  </si>
-  <si>
-    <t>900428482</t>
-  </si>
-  <si>
-    <t>03B900</t>
-  </si>
-  <si>
-    <t>01B303</t>
-  </si>
-  <si>
-    <t>01R064</t>
-  </si>
-  <si>
-    <t>02B538</t>
-  </si>
-  <si>
-    <t>03B079</t>
-  </si>
-  <si>
-    <t>02T130</t>
-  </si>
-  <si>
-    <t>01T555</t>
-  </si>
-  <si>
-    <t>02T680</t>
-  </si>
-  <si>
-    <t>02T597</t>
-  </si>
-  <si>
-    <t>85060</t>
-  </si>
-  <si>
-    <t>104960</t>
-  </si>
-  <si>
-    <t>25960</t>
-  </si>
-  <si>
-    <t>18960</t>
-  </si>
-  <si>
-    <t>139560</t>
-  </si>
-  <si>
-    <t>114260</t>
-  </si>
-  <si>
-    <t>35560</t>
-  </si>
-  <si>
-    <t>30570</t>
-  </si>
-  <si>
-    <t>35960</t>
+    <t>0</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>161503</t>
+  </si>
+  <si>
+    <t>830048991</t>
+  </si>
+  <si>
+    <t>01P456</t>
+  </si>
+  <si>
+    <t>01P759</t>
+  </si>
+  <si>
+    <t>02P389</t>
+  </si>
+  <si>
+    <t>02P598</t>
+  </si>
+  <si>
+    <t>01P032</t>
+  </si>
+  <si>
+    <t>01P409</t>
+  </si>
+  <si>
+    <t>01P320</t>
+  </si>
+  <si>
+    <t>01P036</t>
+  </si>
+  <si>
+    <t>02P047</t>
+  </si>
+  <si>
+    <t>01P031</t>
+  </si>
+  <si>
+    <t>01P692</t>
+  </si>
+  <si>
+    <t>02P326</t>
+  </si>
+  <si>
+    <t>02B242</t>
+  </si>
+  <si>
+    <t>02B715</t>
+  </si>
+  <si>
+    <t>01B442</t>
+  </si>
+  <si>
+    <t>03B089</t>
+  </si>
+  <si>
+    <t>03B519</t>
+  </si>
+  <si>
+    <t>02C932</t>
+  </si>
+  <si>
+    <t>01D396</t>
+  </si>
+  <si>
+    <t>01D322</t>
+  </si>
+  <si>
+    <t>02D004</t>
+  </si>
+  <si>
+    <t>01D385</t>
+  </si>
+  <si>
+    <t>33000</t>
+  </si>
+  <si>
+    <t>25000</t>
+  </si>
+  <si>
+    <t>95000</t>
+  </si>
+  <si>
+    <t>65100</t>
+  </si>
+  <si>
+    <t>30200</t>
+  </si>
+  <si>
+    <t>52200</t>
+  </si>
+  <si>
+    <t>51000</t>
+  </si>
+  <si>
+    <t>52300</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>58000</t>
+  </si>
+  <si>
+    <t>86400</t>
+  </si>
+  <si>
+    <t>78000</t>
+  </si>
+  <si>
+    <t>84900</t>
+  </si>
+  <si>
+    <t>67600</t>
+  </si>
+  <si>
+    <t>60000</t>
+  </si>
+  <si>
+    <t>71000</t>
+  </si>
+  <si>
+    <t>61800</t>
+  </si>
+  <si>
+    <t>84300</t>
+  </si>
+  <si>
+    <t>81500</t>
+  </si>
+  <si>
+    <t>106000</t>
+  </si>
+  <si>
+    <t>94800</t>
+  </si>
+  <si>
+    <t>77500</t>
+  </si>
+  <si>
+    <t>135700</t>
   </si>
 </sst>
 </file>
@@ -263,13 +338,13 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Accent1" xfId="3" builtinId="29"/>
@@ -607,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9761A0BD-3A6E-4B42-BA50-BD0DC4B983CA}">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" style="2" customWidth="1"/>
@@ -619,14 +694,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:12" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -647,58 +722,58 @@
         <v>46272</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>24</v>
-      </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>4</v>
@@ -706,10 +781,10 @@
       <c r="I6">
         <v>2</v>
       </c>
-      <c r="J6" s="6">
+      <c r="J6" s="4">
         <v>266601</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="4">
         <v>442558</v>
       </c>
       <c r="L6">
@@ -719,76 +794,76 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
+      <c r="J8" s="4"/>
+      <c r="K8" s="4"/>
       <c r="L8">
         <v>266</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
+      <c r="J9" s="4"/>
+      <c r="K9" s="4"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>14</v>
@@ -797,16 +872,16 @@
         <v>6</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -816,19 +891,19 @@
         <v>14</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
+      <c r="J11" s="4"/>
+      <c r="K11" s="4"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
@@ -838,19 +913,19 @@
         <v>14</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
@@ -863,16 +938,16 @@
         <v>5</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J13" s="6"/>
-      <c r="K13" s="6"/>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
@@ -882,19 +957,19 @@
         <v>14</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
@@ -907,16 +982,16 @@
         <v>15</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
@@ -929,32 +1004,264 @@
         <v>6</v>
       </c>
       <c r="D16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="J16" s="6"/>
-      <c r="K16" s="6"/>
-    </row>
-    <row r="17" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J17" s="6"/>
-      <c r="K17" s="6"/>
-    </row>
-    <row r="18" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J18" s="6"/>
-      <c r="K18" s="6"/>
-    </row>
-    <row r="19" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
-    </row>
-    <row r="20" spans="10:11" x14ac:dyDescent="0.25">
-      <c r="J20" s="6"/>
-      <c r="K20" s="6"/>
+      <c r="B25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>4</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>